<commit_message>
fixed datasheet, end of day
</commit_message>
<xml_diff>
--- a/data/FirebreakData2026_final.xlsx
+++ b/data/FirebreakData2026_final.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\host.lan\Data\files\tasks\a1f20c73-7c01-4b0e-ab9b-cc46d4c4ec7e\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\host.lan\Data\files\tasks\2e012287-a1b1-49e2-9d2a-b0f7fcdba23b\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{BDEB3670-5D14-45EE-82DE-F1875B9CF4A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{E06D0418-FE3A-460C-A49E-81104F75DA0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="19440" windowHeight="10440"/>
   </bookViews>
@@ -13576,7 +13576,7 @@
         <v>1</v>
       </c>
       <c r="Q4">
-        <v>0.4</v>
+        <v>1</v>
       </c>
       <c r="R4">
         <v>7</v>
@@ -15876,10 +15876,10 @@
       <c r="A82" t="s">
         <v>87</v>
       </c>
-      <c r="P82">
-        <v>1</v>
-      </c>
-      <c r="Q82">
+      <c r="P82" s="1">
+        <v>1</v>
+      </c>
+      <c r="Q82" s="1">
         <v>2</v>
       </c>
     </row>

</xml_diff>